<commit_message>
update UI and highlighting functionality
</commit_message>
<xml_diff>
--- a/assets/dummy_data.xlsx
+++ b/assets/dummy_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\he162696\Documents\ExcelControlCharts\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\he162696\REPOS\ExcelControlCharts\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B90C4CA-ECCD-4D42-9CCF-FEEEA7954A85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1386BD34-3ECC-4697-83F5-EA77D6120D68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-60" yWindow="-60" windowWidth="20640" windowHeight="13200" tabRatio="752" firstSheet="1" activeTab="1" xr2:uid="{B4DE27E6-3CDA-4D86-9B4B-E26F47FA9977}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="752" activeTab="1" xr2:uid="{B4DE27E6-3CDA-4D86-9B4B-E26F47FA9977}"/>
   </bookViews>
   <sheets>
     <sheet name="dummy_data" sheetId="1" r:id="rId1"/>
@@ -957,22 +957,22 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>187325</xdr:colOff>
+      <xdr:colOff>325437</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>153193</xdr:rowOff>
+      <xdr:rowOff>12699</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>190500</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>79374</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>325437</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>12699</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Image">
+        <xdr:cNvPr id="2" name="Image">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{32F734B5-59F4-5617-E721-9B86624FB317}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8595ADDF-F199-DA02-6B55-BDD86B2120F1}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -994,8 +994,208 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2835275" y="1105693"/>
-          <a:ext cx="5489575" cy="4117181"/>
+          <a:off x="2973387" y="965199"/>
+          <a:ext cx="6096000" cy="4572000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>177800</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>31750</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F3CF22D-7110-FFFE-1E2F-B42640A7DF9B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2825750" y="984250"/>
+          <a:ext cx="6096000" cy="4572000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>425450</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>155575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>425450</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>155575</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C87C8559-08B0-D9E4-A2B5-D4CFDCEC3C3F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3073400" y="1298575"/>
+          <a:ext cx="6096000" cy="4572000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>425450</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>425450</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>127000</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Image">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D2AD3AC7-F76E-E14C-E879-ADCA9803B5B2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2463800" y="889000"/>
+          <a:ext cx="6096000" cy="4572000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>1254125</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>117475</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>434975</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>117475</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Image">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C5EB59A2-2BBE-50AB-D552-0EDFE8020326}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId8"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1254125" y="688975"/>
+          <a:ext cx="6096000" cy="4572000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1066,16 +1266,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>463550</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>434975</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>463550</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>184150</xdr:rowOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>434975</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>174625</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1104,7 +1304,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3787775" y="946150"/>
+          <a:off x="3149600" y="746125"/>
           <a:ext cx="6096000" cy="4572000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1121,16 +1321,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>530225</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>98425</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>554038</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>179388</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>530225</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>98425</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>554038</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>179388</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1159,7 +1359,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3835400" y="479425"/>
+          <a:off x="4468813" y="941388"/>
           <a:ext cx="6096000" cy="4572000"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -1463,7 +1663,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0597FC6A-6243-4075-BF4F-A5F3DADF53C9}" name="Table_name_test5" displayName="Table_name_test5" ref="A1:B18" totalsRowShown="0">
   <autoFilter ref="A1:B18" xr:uid="{0597FC6A-6243-4075-BF4F-A5F3DADF53C9}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{DB1E9005-DD79-4D4C-88BC-A9880CDD53AF}" name="Month" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{DB1E9005-DD79-4D4C-88BC-A9880CDD53AF}" name="Month" dataDxfId="11"/>
     <tableColumn id="2" xr3:uid="{C960CA6D-8CFF-48C3-9D74-9D1713E0179A}" name="Events"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1474,7 +1674,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{83B77A84-D877-489A-AC21-D04CD829CB9F}" name="Table_name_test" displayName="Table_name_test" ref="A1:B18" totalsRowShown="0">
   <autoFilter ref="A1:B18" xr:uid="{83B77A84-D877-489A-AC21-D04CD829CB9F}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{53E01FA9-6511-42AB-93B9-1A7BE3AFF00D}" name="Month" dataDxfId="11"/>
+    <tableColumn id="1" xr3:uid="{53E01FA9-6511-42AB-93B9-1A7BE3AFF00D}" name="Month" dataDxfId="10"/>
     <tableColumn id="2" xr3:uid="{0F34ED01-8055-4C38-938D-03F234DD5796}" name="Events"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1488,7 +1688,7 @@
     <sortCondition ref="A1:A18"/>
   </sortState>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{4A712F32-8ECE-4FAB-84FE-6D275F8D1630}" name="Month" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{4A712F32-8ECE-4FAB-84FE-6D275F8D1630}" name="Month" dataDxfId="9"/>
     <tableColumn id="2" xr3:uid="{9A49965A-41A2-4364-8DB1-CAE8F75752E9}" name="Events"/>
     <tableColumn id="3" xr3:uid="{E83D6FC6-367E-40BE-B41E-4F3BA4F2E7EC}" name="Days"/>
   </tableColumns>
@@ -1500,7 +1700,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{E2B1412F-41F0-47E8-9B0E-8E9D0B624679}" name="Table5" displayName="Table5" ref="A1:C18" totalsRowShown="0">
   <autoFilter ref="A1:C18" xr:uid="{E2B1412F-41F0-47E8-9B0E-8E9D0B624679}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{A5EEE1C8-54ED-4A81-AE44-B611E0A76682}" name="Month" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{A5EEE1C8-54ED-4A81-AE44-B611E0A76682}" name="Month" dataDxfId="8"/>
     <tableColumn id="2" xr3:uid="{06FCF3B1-6BEB-4880-88E6-1CD5E8B7A345}" name="Harmed"/>
     <tableColumn id="3" xr3:uid="{C77DF6A1-1AAE-480F-A997-913BB55D23A6}" name="Patients"/>
   </tableColumns>
@@ -1872,7 +2072,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="1158" row="5">
+  <wetp:taskpane dockstate="right" visibility="0" width="606" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -9303,7 +9503,7 @@
         <v>40452</v>
       </c>
       <c r="B11">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -9335,7 +9535,7 @@
         <v>40575</v>
       </c>
       <c r="B15">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -9343,7 +9543,7 @@
         <v>40603</v>
       </c>
       <c r="B16">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -9351,7 +9551,7 @@
         <v>40634</v>
       </c>
       <c r="B17">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -9359,7 +9559,7 @@
         <v>40664</v>
       </c>
       <c r="B18">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>